<commit_message>
update cluster names in figures and supp table 3
</commit_message>
<xml_diff>
--- a/supplementary_tables/SuppTable3_cluster_assignments.xlsx
+++ b/supplementary_tables/SuppTable3_cluster_assignments.xlsx
@@ -632,7 +632,7 @@
     <t xml:space="preserve">1. Innate-to-Adaptive Bridge</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Th1 Effector Hyper-Activation</t>
+    <t xml:space="preserve">2. Th1/Th2 Effector Hyper-Activation</t>
   </si>
   <si>
     <t xml:space="preserve">3. Exhaustion &amp; Chronic Inflammation</t>
@@ -644,28 +644,28 @@
     <t xml:space="preserve">5. Myeloid Resolution Failure</t>
   </si>
   <si>
-    <t xml:space="preserve">6. Dysregulated Repair Timing</t>
+    <t xml:space="preserve">6. Dysregulated Repair</t>
   </si>
   <si>
     <t xml:space="preserve">IL17F</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Early Neuro-Vascular Surge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Systemic Exhaustion &amp; Barrier Stress</t>
+    <t xml:space="preserve">1. Effector Cytokine &amp; Chemokine Activation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Exhaustion &amp; Chronic Inflammation</t>
   </si>
   <si>
     <t xml:space="preserve">3. Immune Checkpoint &amp; Myeloid Remodeling</t>
   </si>
   <si>
-    <t xml:space="preserve">4. Persistent Neuro-Inflammation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. Homeostatic &amp; Niche Suppression</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6. Innate Recruitment &amp; Neuro-Recovery Failure</t>
+    <t xml:space="preserve">4. Neuroinflammation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. Niche Homeostasis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. Neuro-Recovery Failure</t>
   </si>
   <si>
     <t xml:space="preserve">1. Early Chemotaxis &amp; Innate Priming</t>
@@ -674,7 +674,7 @@
     <t xml:space="preserve">2. The Effector Engine</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Antigen Presentation &amp; Th1 Readiness</t>
+    <t xml:space="preserve">3. Interferons &amp; Cytotoxicity</t>
   </si>
   <si>
     <t xml:space="preserve">4. Exhaustion Management</t>

</xml_diff>